<commit_message>
identity instead of intersect, option to ignore pest disturbance
</commit_message>
<xml_diff>
--- a/Documentation/ComparisonofAllMethods.xlsx
+++ b/Documentation/ComparisonofAllMethods.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bcgov-my.sharepoint.com/personal/jennifer_marr_gov_bc_ca/Documents/Working/ECA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\bctsdata\data\north_root\Library\Scripts\ECA\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="589" documentId="8_{4185DEA5-F55A-42B4-B963-72C26BD5EA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7977E14F-C709-450B-81EF-EEDEAD154938}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Process" sheetId="5" r:id="rId1"/>

</xml_diff>

<commit_message>
comment out pest and vri, update field for watersheds with subbasins, updated comparison of all methods spreadsheet, added recovery curves, delete old tbx and add new one
</commit_message>
<xml_diff>
--- a/Documentation/ComparisonofAllMethods.xlsx
+++ b/Documentation/ComparisonofAllMethods.xlsx
@@ -5,16 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\bctsdata\data\north_root\Library\Scripts\ECA\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\north_root\Library\Scripts\ECA\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="589" documentId="8_{4185DEA5-F55A-42B4-B963-72C26BD5EA6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7977E14F-C709-450B-81EF-EEDEAD154938}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE97F7BF-026E-4039-9E6B-BDF46F4464B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Process" sheetId="5" r:id="rId1"/>
     <sheet name="Data Sources" sheetId="2" r:id="rId2"/>
+    <sheet name="Recovery Curves" sheetId="6" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_Toc199171415" localSheetId="0">'Current Process'!#REF!</definedName>
@@ -82,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="122">
   <si>
     <t>Foresite</t>
   </si>
@@ -167,9 +168,6 @@
     <t>Room for Improvement</t>
   </si>
   <si>
-    <t>Use LiDAR to estimate CHM and extrapolate growth since acquisition date</t>
-  </si>
-  <si>
     <t>Comments</t>
   </si>
   <si>
@@ -352,9 +350,6 @@
     <t xml:space="preserve">Increases ECA values </t>
   </si>
   <si>
-    <t>Increases ECA values</t>
-  </si>
-  <si>
     <t>Private land is 75% ECA</t>
   </si>
   <si>
@@ -447,13 +442,63 @@
   </si>
   <si>
     <t>is this results?</t>
+  </si>
+  <si>
+    <t>removed - April 23 2026</t>
+  </si>
+  <si>
+    <t>chose not to include these as of April 2026, since they don't necessarily mean disturbance.  Could be shorter stands due to elevation, sandy/rock soil.  Remote sensing data unreliable</t>
+  </si>
+  <si>
+    <t>Winkler, R. and S. Boon, 2015. Revised snow recovery estimates for pine-dominated forests in interior British Columbia. Province of B.C., Victoria, B.C.</t>
+  </si>
+  <si>
+    <t>Available from:</t>
+  </si>
+  <si>
+    <t>http://www.for.gov.bc.ca/hfd/pubs/docs/en/EN116.PDF [Accessed 29 Oct 2024]</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Provincial Aquatic Ecosystems Technical Working Group – Ministry of Environment and Climate Change Strategy and Ministry of Forests, Lands and Natural Resource Operations and Rural Development, December 2020. </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Interim Assessment Protocol for Aquatic Ecosystems in British Columbia – Standards for Assessing the Condition of Aquatic Ecosystems under British Columbia’s Cumulative Effects Framework</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. Available from:</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www2.gov.bc.ca/assets/gov/environment/natural-resource-stewardship/cumulative-effects/protocols/cef-aquatic-ecosystems-protocol-dec2020.pdf  [Accessed 29 Oct 2024]</t>
+  </si>
+  <si>
+    <t>site_index &gt;= 12 --&gt; 25m height expectancy</t>
+  </si>
+  <si>
+    <t>site_index &lt; 12 --&gt; 20m heigh expectancy</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -526,6 +571,67 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="5.5"/>
+      <color theme="0" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="5.5"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -557,7 +663,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -665,24 +771,14 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </left>
-      <right style="thin">
-        <color theme="0" tint="-0.34998626667073579"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -753,8 +849,29 @@
     <xf numFmtId="9" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="11" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -774,9 +891,12 @@
     <xf numFmtId="9" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="2" builtinId="10"/>
   </cellStyles>
@@ -970,6 +1090,116 @@
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>198120</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>45720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>156845</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>166370</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2" descr="A white rectangular object with black lines&#10;&#10;Description automatically generated">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F48B7CB-E96D-60EE-5786-1D67E6299B8A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6294120" y="8641080"/>
+          <a:ext cx="4225925" cy="1217930"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>160020</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>115158</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>83820</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B0CA1258-EA5A-8BA0-BD11-86A1DE266D7D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="304800" y="160020"/>
+          <a:ext cx="10783158" cy="6690360"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -1343,25 +1573,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
     </row>
     <row r="2" spans="2:12" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
     </row>
     <row r="4" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1"/>
@@ -1384,23 +1614,23 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>25</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K6" s="18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="38" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -1417,11 +1647,11 @@
         <v>10</v>
       </c>
       <c r="L7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="2:12" ht="121.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="31"/>
+      <c r="B8" s="38"/>
       <c r="C8" s="6" t="s">
         <v>7</v>
       </c>
@@ -1429,20 +1659,20 @@
         <v>12</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>10</v>
       </c>
       <c r="L8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="31"/>
+      <c r="B9" s="38"/>
       <c r="C9" s="8" t="s">
         <v>8</v>
       </c>
@@ -1457,28 +1687,28 @@
         <v>10</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B10" s="31"/>
+      <c r="B10" s="38"/>
       <c r="C10" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D10" s="8"/>
       <c r="E10" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="K10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B11" s="31"/>
+      <c r="B11" s="38"/>
       <c r="C11" s="6" t="s">
         <v>4</v>
       </c>
@@ -1493,68 +1723,66 @@
         <v>10</v>
       </c>
       <c r="K11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="2:12" ht="93" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="31"/>
+      <c r="B12" s="38"/>
       <c r="C12" s="6" t="s">
         <v>24</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B13" s="31"/>
+    <row r="13" spans="2:12" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="38"/>
       <c r="C13" s="6" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="8"/>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="F13" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>10</v>
+      <c r="F13" s="6"/>
+      <c r="G13" s="9" t="s">
+        <v>114</v>
       </c>
       <c r="K13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="2:12" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B14" s="31"/>
+      <c r="B14" s="38"/>
       <c r="C14" s="6" t="s">
         <v>23</v>
       </c>
       <c r="D14" s="8"/>
-      <c r="E14" s="5" t="s">
-        <v>66</v>
+      <c r="E14" s="31" t="s">
+        <v>65</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="9" t="s">
-        <v>83</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B15" s="31"/>
+      <c r="B15" s="38"/>
       <c r="C15" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="8"/>
       <c r="E15" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F15" s="8"/>
       <c r="G15" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
@@ -1572,7 +1800,7 @@
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="2:12" x14ac:dyDescent="0.3">
@@ -1580,13 +1808,13 @@
         <v>17</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F17" s="17"/>
       <c r="G17" s="7" t="s">
@@ -1601,7 +1829,7 @@
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="K18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="19" spans="2:12" ht="247.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1648,20 +1876,20 @@
         <v>121.71</v>
       </c>
       <c r="L21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" spans="2:12" x14ac:dyDescent="0.3">
       <c r="J23" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="K23" s="20" t="s">
         <v>56</v>
-      </c>
-      <c r="K23" s="20" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.3">
       <c r="J24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K24" s="21">
         <v>0</v>
@@ -1669,7 +1897,7 @@
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.3">
       <c r="J25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K25" s="21">
         <v>25</v>
@@ -1677,7 +1905,7 @@
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.3">
       <c r="J26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="K26" s="21">
         <v>50</v>
@@ -1685,7 +1913,7 @@
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.3">
       <c r="J27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K27" s="21">
         <v>75</v>
@@ -1693,7 +1921,7 @@
     </row>
     <row r="28" spans="2:12" x14ac:dyDescent="0.3">
       <c r="J28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="K28" s="21">
         <v>90</v>
@@ -1728,19 +1956,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C1" s="25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D1" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="25" t="s">
         <v>41</v>
-      </c>
-      <c r="E1" s="25" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1751,324 +1979,335 @@
         <v>0.75</v>
       </c>
       <c r="C2" s="27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D2" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E2" s="26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B3" s="27">
         <v>1</v>
       </c>
       <c r="C3" s="27" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="E3" s="26" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="40">
+        <v>1</v>
+      </c>
+      <c r="C4" s="41" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="E4" s="26" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="39"/>
+      <c r="B5" s="40"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="26" t="s">
+        <v>93</v>
+      </c>
+      <c r="E5" s="26"/>
+    </row>
+    <row r="6" spans="1:5" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="39"/>
+      <c r="B6" s="40"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="26"/>
+    </row>
+    <row r="7" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="39"/>
+      <c r="B7" s="40"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="26" t="s">
+        <v>95</v>
+      </c>
+      <c r="E7" s="26"/>
+    </row>
+    <row r="8" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="39"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="26" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="26"/>
+    </row>
+    <row r="9" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="39"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="26" t="s">
+        <v>97</v>
+      </c>
+      <c r="E9" s="26"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="39" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="40">
+        <v>1</v>
+      </c>
+      <c r="C10" s="41" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="26" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="26" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="39"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="E11" s="26"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="39" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="40">
+        <v>1</v>
+      </c>
+      <c r="C12" s="41" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="26" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="39"/>
+      <c r="B13" s="40"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="E13" s="26" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="39"/>
+      <c r="B14" s="40"/>
+      <c r="C14" s="41"/>
+      <c r="D14" s="26" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="26"/>
+    </row>
+    <row r="15" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="39"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="41"/>
+      <c r="D15" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="E15" s="26"/>
+    </row>
+    <row r="16" spans="1:5" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="39"/>
+      <c r="B16" s="40"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="26" t="s">
+        <v>104</v>
+      </c>
+      <c r="E16" s="26"/>
+    </row>
+    <row r="17" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="39"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="41"/>
+      <c r="D17" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="39"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="26" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="26" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="D3" s="26" t="s">
-        <v>72</v>
-      </c>
-      <c r="E3" s="26" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="32" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="33">
-        <v>1</v>
-      </c>
-      <c r="C4" s="34" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="E4" s="26" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="32"/>
-      <c r="B5" s="33"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="26" t="s">
-        <v>95</v>
-      </c>
-      <c r="E5" s="26"/>
-    </row>
-    <row r="6" spans="1:5" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="32"/>
-      <c r="B6" s="33"/>
-      <c r="C6" s="34"/>
-      <c r="D6" s="26" t="s">
-        <v>96</v>
-      </c>
-      <c r="E6" s="26"/>
-    </row>
-    <row r="7" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="32"/>
-      <c r="B7" s="33"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="26" t="s">
-        <v>97</v>
-      </c>
-      <c r="E7" s="26"/>
-    </row>
-    <row r="8" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="32"/>
-      <c r="B8" s="33"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="26" t="s">
-        <v>98</v>
-      </c>
-      <c r="E8" s="26"/>
-    </row>
-    <row r="9" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="32"/>
-      <c r="B9" s="33"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="26" t="s">
-        <v>99</v>
-      </c>
-      <c r="E9" s="26"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="32" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="33">
-        <v>1</v>
-      </c>
-      <c r="C10" s="34" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="E10" s="26" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="16.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="32"/>
-      <c r="B11" s="33"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="26" t="s">
-        <v>110</v>
-      </c>
-      <c r="E11" s="26"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="33">
-        <v>1</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" s="26" t="s">
-        <v>100</v>
-      </c>
-      <c r="E12" s="26" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="32"/>
-      <c r="B13" s="33"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="26" t="s">
-        <v>103</v>
-      </c>
-      <c r="E13" s="26" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="32"/>
-      <c r="B14" s="33"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="E14" s="26"/>
-    </row>
-    <row r="15" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="32"/>
-      <c r="B15" s="33"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="E15" s="26"/>
-    </row>
-    <row r="16" spans="1:5" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="32"/>
-      <c r="B16" s="33"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="26" t="s">
-        <v>106</v>
-      </c>
-      <c r="E16" s="26"/>
-    </row>
-    <row r="17" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="32"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="26" t="s">
-        <v>107</v>
-      </c>
-      <c r="E17" s="26" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="32"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="E18" s="26" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="27" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="C19" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="D19" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" s="26"/>
+      <c r="D19" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="E19" s="28"/>
+      <c r="F19" s="23" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C20" s="27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D20" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="E20" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="E20" s="26" t="s">
-        <v>75</v>
-      </c>
+      <c r="F20" s="23"/>
     </row>
     <row r="21" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A21" s="26" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="26" t="s">
-        <v>44</v>
-      </c>
       <c r="C21" s="27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D21" s="26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E21" s="26" t="s">
-        <v>50</v>
-      </c>
-      <c r="F21" s="28" t="s">
-        <v>114</v>
+        <v>49</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="D22" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="26" t="s">
-        <v>65</v>
-      </c>
-      <c r="C22" s="27" t="s">
-        <v>55</v>
-      </c>
-      <c r="D22" s="26" t="s">
-        <v>46</v>
-      </c>
       <c r="E22" s="26"/>
+      <c r="F22" s="23"/>
     </row>
     <row r="23" spans="1:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B23" s="27">
         <v>1</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E23" s="26"/>
+      <c r="F23" s="23"/>
     </row>
     <row r="24" spans="1:6" ht="19.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B24" s="27">
         <v>1</v>
       </c>
       <c r="C24" s="27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E24" s="26"/>
+      <c r="F24" s="23"/>
     </row>
     <row r="25" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A25" s="27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B25" s="27">
         <v>1</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D25" s="26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E25" s="26"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="26" t="s">
+      <c r="F25" s="23"/>
+    </row>
+    <row r="26" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="26" t="s">
+      <c r="C26" s="30" t="s">
+        <v>86</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>88</v>
+      </c>
+      <c r="E26" s="28" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="27" t="s">
-        <v>88</v>
-      </c>
-      <c r="D26" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="E26" s="26" t="s">
-        <v>91</v>
+      <c r="F26" s="23" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -2098,4 +2337,90 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3723A69-0912-45A6-B501-EE3AE869014A}">
+  <dimension ref="A27:T46"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="27" spans="20:20" x14ac:dyDescent="0.3">
+      <c r="T27" s="42" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="28" spans="20:20" x14ac:dyDescent="0.3">
+      <c r="T28" s="43" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A40" s="35" t="s">
+        <v>115</v>
+      </c>
+      <c r="B40" s="35"/>
+      <c r="C40" s="35"/>
+      <c r="D40" s="35"/>
+      <c r="E40" s="35"/>
+      <c r="F40" s="35"/>
+      <c r="G40" s="35"/>
+      <c r="H40" s="35"/>
+      <c r="I40" s="35"/>
+      <c r="J40" s="35"/>
+      <c r="K40" s="35"/>
+      <c r="L40" s="35"/>
+      <c r="M40" s="35"/>
+      <c r="N40" s="35"/>
+      <c r="O40" s="35"/>
+      <c r="P40" s="35"/>
+      <c r="Q40" s="35"/>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A41" s="32" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A42" s="33" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="B45" s="34"/>
+      <c r="C45" s="34"/>
+      <c r="D45" s="34"/>
+      <c r="E45" s="34"/>
+      <c r="F45" s="34"/>
+      <c r="G45" s="34"/>
+      <c r="H45" s="34"/>
+      <c r="I45" s="34"/>
+      <c r="J45" s="34"/>
+      <c r="K45" s="34"/>
+      <c r="L45" s="34"/>
+      <c r="M45" s="34"/>
+      <c r="N45" s="34"/>
+      <c r="O45" s="34"/>
+      <c r="P45" s="34"/>
+      <c r="Q45" s="34"/>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A46" s="33" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A45:Q45"/>
+    <mergeCell ref="A40:Q40"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A42" r:id="rId1" display="http://www.for.gov.bc.ca/hfd/pubs/docs/en/EN116.PDF" xr:uid="{8F22B2C4-5CF5-4A99-AED1-3C8480BA46A4}"/>
+    <hyperlink ref="A46" r:id="rId2" display="https://www2.gov.bc.ca/assets/gov/environment/natural-resource-stewardship/cumulative-effects/protocols/cef-aquatic-ecosystems-protocol-dec2020.pdf" xr:uid="{240B1041-6E14-49DB-8BC9-201DA323B42E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add RG to BCTS blocks
</commit_message>
<xml_diff>
--- a/Documentation/ComparisonofAllMethods.xlsx
+++ b/Documentation/ComparisonofAllMethods.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\north_root\Library\Scripts\ECA\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1C33EA-5FA2-4380-8D5D-1A4C6374372C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A72EF4-02BA-4F43-966B-05893C3883BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Process" sheetId="5" r:id="rId1"/>
@@ -872,29 +872,29 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1576,25 +1576,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
     </row>
     <row r="2" spans="2:12" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="37" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="39"/>
-      <c r="G3" s="39"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
     </row>
     <row r="4" spans="2:12" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="1"/>
@@ -1633,7 +1633,7 @@
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="38" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="3" t="s">
@@ -1654,7 +1654,7 @@
       </c>
     </row>
     <row r="8" spans="2:12" ht="121.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="40"/>
+      <c r="B8" s="38"/>
       <c r="C8" s="6" t="s">
         <v>7</v>
       </c>
@@ -1675,7 +1675,7 @@
       </c>
     </row>
     <row r="9" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B9" s="40"/>
+      <c r="B9" s="38"/>
       <c r="C9" s="8" t="s">
         <v>8</v>
       </c>
@@ -1694,7 +1694,7 @@
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B10" s="40"/>
+      <c r="B10" s="38"/>
       <c r="C10" s="6" t="s">
         <v>29</v>
       </c>
@@ -1711,7 +1711,7 @@
       </c>
     </row>
     <row r="11" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B11" s="40"/>
+      <c r="B11" s="38"/>
       <c r="C11" s="6" t="s">
         <v>4</v>
       </c>
@@ -1730,7 +1730,7 @@
       </c>
     </row>
     <row r="12" spans="2:12" ht="93" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="40"/>
+      <c r="B12" s="38"/>
       <c r="C12" s="6" t="s">
         <v>24</v>
       </c>
@@ -1744,7 +1744,7 @@
       </c>
     </row>
     <row r="13" spans="2:12" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="40"/>
+      <c r="B13" s="38"/>
       <c r="C13" s="6" t="s">
         <v>6</v>
       </c>
@@ -1761,7 +1761,7 @@
       </c>
     </row>
     <row r="14" spans="2:12" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B14" s="40"/>
+      <c r="B14" s="38"/>
       <c r="C14" s="6" t="s">
         <v>23</v>
       </c>
@@ -1775,7 +1775,7 @@
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B15" s="40"/>
+      <c r="B15" s="38"/>
       <c r="C15" s="8" t="s">
         <v>9</v>
       </c>
@@ -2009,13 +2009,13 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="42">
+      <c r="B4" s="40">
         <v>1</v>
       </c>
-      <c r="C4" s="43" t="s">
+      <c r="C4" s="41" t="s">
         <v>53</v>
       </c>
       <c r="D4" s="26" t="s">
@@ -2026,58 +2026,58 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="41"/>
-      <c r="B5" s="42"/>
-      <c r="C5" s="43"/>
+      <c r="A5" s="39"/>
+      <c r="B5" s="40"/>
+      <c r="C5" s="41"/>
       <c r="D5" s="26" t="s">
         <v>93</v>
       </c>
       <c r="E5" s="26"/>
     </row>
     <row r="6" spans="1:5" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="41"/>
-      <c r="B6" s="42"/>
-      <c r="C6" s="43"/>
+      <c r="A6" s="39"/>
+      <c r="B6" s="40"/>
+      <c r="C6" s="41"/>
       <c r="D6" s="26" t="s">
         <v>94</v>
       </c>
       <c r="E6" s="26"/>
     </row>
     <row r="7" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="41"/>
-      <c r="B7" s="42"/>
-      <c r="C7" s="43"/>
+      <c r="A7" s="39"/>
+      <c r="B7" s="40"/>
+      <c r="C7" s="41"/>
       <c r="D7" s="26" t="s">
         <v>95</v>
       </c>
       <c r="E7" s="26"/>
     </row>
     <row r="8" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="41"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="43"/>
+      <c r="A8" s="39"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="41"/>
       <c r="D8" s="26" t="s">
         <v>96</v>
       </c>
       <c r="E8" s="26"/>
     </row>
     <row r="9" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="41"/>
-      <c r="B9" s="42"/>
-      <c r="C9" s="43"/>
+      <c r="A9" s="39"/>
+      <c r="B9" s="40"/>
+      <c r="C9" s="41"/>
       <c r="D9" s="26" t="s">
         <v>97</v>
       </c>
       <c r="E9" s="26"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="42">
+      <c r="B10" s="40">
         <v>1</v>
       </c>
-      <c r="C10" s="43" t="s">
+      <c r="C10" s="41" t="s">
         <v>53</v>
       </c>
       <c r="D10" s="26" t="s">
@@ -2088,22 +2088,22 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="16.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="41"/>
-      <c r="B11" s="42"/>
-      <c r="C11" s="43"/>
+      <c r="A11" s="39"/>
+      <c r="B11" s="40"/>
+      <c r="C11" s="41"/>
       <c r="D11" s="26" t="s">
         <v>108</v>
       </c>
       <c r="E11" s="26"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="41" t="s">
+      <c r="A12" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="42">
+      <c r="B12" s="40">
         <v>1</v>
       </c>
-      <c r="C12" s="43" t="s">
+      <c r="C12" s="41" t="s">
         <v>53</v>
       </c>
       <c r="D12" s="26" t="s">
@@ -2114,9 +2114,9 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="41"/>
-      <c r="B13" s="42"/>
-      <c r="C13" s="43"/>
+      <c r="A13" s="39"/>
+      <c r="B13" s="40"/>
+      <c r="C13" s="41"/>
       <c r="D13" s="26" t="s">
         <v>101</v>
       </c>
@@ -2125,36 +2125,36 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="41"/>
-      <c r="B14" s="42"/>
-      <c r="C14" s="43"/>
+      <c r="A14" s="39"/>
+      <c r="B14" s="40"/>
+      <c r="C14" s="41"/>
       <c r="D14" s="26" t="s">
         <v>102</v>
       </c>
       <c r="E14" s="26"/>
     </row>
     <row r="15" spans="1:5" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="41"/>
-      <c r="B15" s="42"/>
-      <c r="C15" s="43"/>
+      <c r="A15" s="39"/>
+      <c r="B15" s="40"/>
+      <c r="C15" s="41"/>
       <c r="D15" s="26" t="s">
         <v>103</v>
       </c>
       <c r="E15" s="26"/>
     </row>
     <row r="16" spans="1:5" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="41"/>
-      <c r="B16" s="42"/>
-      <c r="C16" s="43"/>
+      <c r="A16" s="39"/>
+      <c r="B16" s="40"/>
+      <c r="C16" s="41"/>
       <c r="D16" s="26" t="s">
         <v>104</v>
       </c>
       <c r="E16" s="26"/>
     </row>
     <row r="17" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="41"/>
-      <c r="B17" s="42"/>
-      <c r="C17" s="43"/>
+      <c r="A17" s="39"/>
+      <c r="B17" s="40"/>
+      <c r="C17" s="41"/>
       <c r="D17" s="26" t="s">
         <v>105</v>
       </c>
@@ -2163,9 +2163,9 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="41"/>
-      <c r="B18" s="42"/>
-      <c r="C18" s="43"/>
+      <c r="A18" s="39"/>
+      <c r="B18" s="40"/>
+      <c r="C18" s="41"/>
       <c r="D18" s="26" t="s">
         <v>90</v>
       </c>
@@ -2173,7 +2173,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="46.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="2.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="29" t="s">
         <v>27</v>
       </c>
@@ -2209,7 +2209,7 @@
       </c>
       <c r="F20" s="23"/>
     </row>
-    <row r="21" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="26" t="s">
         <v>42</v>
       </c>
@@ -2293,7 +2293,7 @@
       <c r="E25" s="26"/>
       <c r="F25" s="23"/>
     </row>
-    <row r="26" spans="1:6" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" ht="1.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="30" t="s">
         <v>85</v>
       </c>
@@ -2358,25 +2358,25 @@
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A40" s="37" t="s">
+      <c r="A40" s="43" t="s">
         <v>115</v>
       </c>
-      <c r="B40" s="37"/>
-      <c r="C40" s="37"/>
-      <c r="D40" s="37"/>
-      <c r="E40" s="37"/>
-      <c r="F40" s="37"/>
-      <c r="G40" s="37"/>
-      <c r="H40" s="37"/>
-      <c r="I40" s="37"/>
-      <c r="J40" s="37"/>
-      <c r="K40" s="37"/>
-      <c r="L40" s="37"/>
-      <c r="M40" s="37"/>
-      <c r="N40" s="37"/>
-      <c r="O40" s="37"/>
-      <c r="P40" s="37"/>
-      <c r="Q40" s="37"/>
+      <c r="B40" s="43"/>
+      <c r="C40" s="43"/>
+      <c r="D40" s="43"/>
+      <c r="E40" s="43"/>
+      <c r="F40" s="43"/>
+      <c r="G40" s="43"/>
+      <c r="H40" s="43"/>
+      <c r="I40" s="43"/>
+      <c r="J40" s="43"/>
+      <c r="K40" s="43"/>
+      <c r="L40" s="43"/>
+      <c r="M40" s="43"/>
+      <c r="N40" s="43"/>
+      <c r="O40" s="43"/>
+      <c r="P40" s="43"/>
+      <c r="Q40" s="43"/>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A41" s="32" t="s">
@@ -2389,25 +2389,25 @@
       </c>
     </row>
     <row r="45" spans="1:17" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="36" t="s">
+      <c r="A45" s="42" t="s">
         <v>118</v>
       </c>
-      <c r="B45" s="36"/>
-      <c r="C45" s="36"/>
-      <c r="D45" s="36"/>
-      <c r="E45" s="36"/>
-      <c r="F45" s="36"/>
-      <c r="G45" s="36"/>
-      <c r="H45" s="36"/>
-      <c r="I45" s="36"/>
-      <c r="J45" s="36"/>
-      <c r="K45" s="36"/>
-      <c r="L45" s="36"/>
-      <c r="M45" s="36"/>
-      <c r="N45" s="36"/>
-      <c r="O45" s="36"/>
-      <c r="P45" s="36"/>
-      <c r="Q45" s="36"/>
+      <c r="B45" s="42"/>
+      <c r="C45" s="42"/>
+      <c r="D45" s="42"/>
+      <c r="E45" s="42"/>
+      <c r="F45" s="42"/>
+      <c r="G45" s="42"/>
+      <c r="H45" s="42"/>
+      <c r="I45" s="42"/>
+      <c r="J45" s="42"/>
+      <c r="K45" s="42"/>
+      <c r="L45" s="42"/>
+      <c r="M45" s="42"/>
+      <c r="N45" s="42"/>
+      <c r="O45" s="42"/>
+      <c r="P45" s="42"/>
+      <c r="Q45" s="42"/>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A46" s="33" t="s">

</xml_diff>